<commit_message>
Re-ingest crosswalk: Safeway IMW now totals Denver + Intermountain
Updated Nielsen_crosswalk.xlsx maps the Safeway IMW sales account to
both the ALBSCO Denver Div TA and the Intermountain Div TA, so scoping
to IMW totals the two divisions; the standalone Safeway Denver account
remains for Denver alone. The ingest script gains an exact-duplicate
guard (the update carried a doubled IMW -> Intermountain row, dropped
with a warning). All 14 loaded market rows resolve; parent ALBSCO still
dedupes to 13 distinct divisions.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X7uiPtQBdfYJKyK6vHm2QA
</commit_message>
<xml_diff>
--- a/data/raw/Nielsen_crosswalk.xlsx
+++ b/data/raw/Nielsen_crosswalk.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7f067a049cfb567a/Documents/Heartland/Crosswalk Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{4FD583A2-48CF-48EF-8A2C-EDE4FDBD2DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE420AE4-6158-4746-B60F-E3D170E3D7E5}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{4FD583A2-48CF-48EF-8A2C-EDE4FDBD2DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7D02A56-71DB-4D54-B581-8EECE3A2E324}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C34369D8-7A71-41E5-BE42-3F2A05B0E4D3}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C34369D8-7A71-41E5-BE42-3F2A05B0E4D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Reporting Tab" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reporting Tab'!$A$6:$H$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reporting Tab'!$A$6:$H$84</definedName>
     <definedName name="Chockys_Hot_Cocoa_Liquid_Pods">[1]!Table394142[Liquid_Pods]</definedName>
     <definedName name="Equal_Creamers_Bottles_50mL">[1]!Table53[Bottles_50mL]</definedName>
     <definedName name="Equal_Sweeteners_Aspartame">[1]!Table50[Aspartame]</definedName>
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="193">
   <si>
     <t>Customer Name</t>
   </si>
@@ -1144,6 +1144,10 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1325,7 +1329,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B742A881-8B70-4CE1-B28B-3A10AD0129F6}">
-  <dimension ref="A2:H82"/>
+  <dimension ref="A2:H84"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.6640625" customWidth="1"/>
@@ -2883,7 +2887,7 @@
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>6</v>
@@ -2892,72 +2896,76 @@
         <v>146</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>184</v>
+        <v>163</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F67" s="4" t="s">
         <v>148</v>
       </c>
       <c r="G67" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="H67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F68" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="H67" s="4" t="s">
+      <c r="G68" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="H68" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A69" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="H69" s="4" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A68" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C68" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="D68" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="E68" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="F68" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="G68" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="H68" s="6"/>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A69" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C69" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="E69" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="F69" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="G69" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="H69" s="6"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>6</v>
@@ -2969,7 +2977,7 @@
         <v>175</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F70" s="4" t="s">
         <v>137</v>
@@ -2981,31 +2989,31 @@
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>74</v>
+        <v>185</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="H71" s="6"/>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>6</v>
@@ -3017,7 +3025,7 @@
         <v>175</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F72" s="4" t="s">
         <v>137</v>
@@ -3029,103 +3037,103 @@
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>186</v>
+        <v>74</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="G73" s="4" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="H73" s="6"/>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="H74" s="6"/>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="G75" s="4" t="s">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="H75" s="6"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="H76" s="6"/>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B77" s="3" t="s">
         <v>6</v>
@@ -3134,22 +3142,22 @@
         <v>146</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>163</v>
+        <v>188</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F77" s="4" t="s">
         <v>148</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="H77" s="6"/>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>6</v>
@@ -3158,10 +3166,10 @@
         <v>136</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F78" s="4" t="s">
         <v>137</v>
@@ -3173,19 +3181,19 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B79" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>190</v>
+        <v>146</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>163</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F79" s="4" t="s">
         <v>148</v>
@@ -3197,7 +3205,7 @@
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B80" s="3" t="s">
         <v>6</v>
@@ -3209,7 +3217,7 @@
         <v>175</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F80" s="4" t="s">
         <v>137</v>
@@ -3221,54 +3229,102 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B81" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>136</v>
+        <v>190</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>191</v>
+        <v>163</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="H81" s="6"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="E82" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F82" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="G82" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="H82" s="6"/>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A83" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="E83" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="F83" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="G83" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="H83" s="6"/>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A84" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B82" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C82" s="4" t="s">
+      <c r="B84" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C84" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="D82" s="4" t="s">
+      <c r="D84" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E82" s="4" t="s">
+      <c r="E84" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F82" s="4" t="s">
+      <c r="F84" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="G82" s="4" t="s">
+      <c r="G84" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="H82" s="6"/>
+      <c r="H84" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A6:H82" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A6:H84" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>